<commit_message>
feat: overhaul furniture placement backgrounds grids and scale
</commit_message>
<xml_diff>
--- a/Excel/家具房间表.xlsx
+++ b/Excel/家具房间表.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="房间" sheetId="1" r:id="Rbdd714245fb44674"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网格" sheetId="2" r:id="Rec60b807645a4e58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="占用格" sheetId="3" r:id="R25e5b29dac714813"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初始摆放" sheetId="4" r:id="R6b9718284f244760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="房间" sheetId="1" r:id="R189b7194a6704bed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网格" sheetId="2" r:id="R78b438265b7448e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="占用格" sheetId="3" r:id="R859aedb57e0d4072"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初始摆放" sheetId="4" r:id="R8884564ef8e2478e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -968,16 +968,16 @@
         </x:is>
       </x:c>
       <x:c r="D3" t="n">
-        <x:v>34</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E3" t="n">
-        <x:v>14</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F3" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G3" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H3" t="n">
         <x:v>316</x:v>
@@ -1006,19 +1006,19 @@
         </x:is>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>53</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E4" t="n">
-        <x:v>5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F4" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G4" t="n">
-        <x:v>21.6</x:v>
+        <x:v>10.8</x:v>
       </x:c>
       <x:c r="H4" t="n">
-        <x:v>40</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I4" t="n">
         <x:v>500</x:v>
@@ -1044,16 +1044,16 @@
         </x:is>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>28</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:v>13</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F5" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G5" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H5" t="n">
         <x:v>242</x:v>
@@ -1082,19 +1082,19 @@
         </x:is>
       </x:c>
       <x:c r="D6" t="n">
-        <x:v>53</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E6" t="n">
-        <x:v>4</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F6" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G6" t="n">
-        <x:v>21</x:v>
+        <x:v>10.5</x:v>
       </x:c>
       <x:c r="H6" t="n">
-        <x:v>40</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I6" t="n">
         <x:v>530</x:v>
@@ -1120,16 +1120,16 @@
         </x:is>
       </x:c>
       <x:c r="D7" t="n">
-        <x:v>24</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E7" t="n">
-        <x:v>14</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F7" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G7" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H7" t="n">
         <x:v>562</x:v>
@@ -1158,19 +1158,19 @@
         </x:is>
       </x:c>
       <x:c r="D8" t="n">
-        <x:v>53</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E8" t="n">
-        <x:v>5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F8" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G8" t="n">
-        <x:v>20.8</x:v>
+        <x:v>10.4</x:v>
       </x:c>
       <x:c r="H8" t="n">
-        <x:v>40</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I8" t="n">
         <x:v>502</x:v>
@@ -1196,16 +1196,16 @@
         </x:is>
       </x:c>
       <x:c r="D9" t="n">
-        <x:v>46</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E9" t="n">
-        <x:v>14</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F9" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G9" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H9" t="n">
         <x:v>130</x:v>
@@ -1234,19 +1234,19 @@
         </x:is>
       </x:c>
       <x:c r="D10" t="n">
-        <x:v>53</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E10" t="n">
-        <x:v>5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F10" t="n">
-        <x:v>30</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G10" t="n">
-        <x:v>20.1</x:v>
+        <x:v>10.05</x:v>
       </x:c>
       <x:c r="H10" t="n">
-        <x:v>40</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="I10" t="n">
         <x:v>502</x:v>
@@ -1417,10 +1417,10 @@
         </x:is>
       </x:c>
       <x:c r="E3" t="n">
-        <x:v>8</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F3" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G3" t="inlineStr">
         <x:is>
@@ -1445,10 +1445,10 @@
         </x:is>
       </x:c>
       <x:c r="E4" t="n">
-        <x:v>25</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F4" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G4" t="inlineStr">
         <x:is>
@@ -1473,10 +1473,10 @@
         </x:is>
       </x:c>
       <x:c r="E5" t="n">
-        <x:v>17</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F5" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G5" t="inlineStr">
         <x:is>
@@ -1501,10 +1501,10 @@
         </x:is>
       </x:c>
       <x:c r="E6" t="n">
-        <x:v>25</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F6" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G6" t="inlineStr">
         <x:is>
@@ -1529,10 +1529,10 @@
         </x:is>
       </x:c>
       <x:c r="E7" t="n">
-        <x:v>16</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F7" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G7" t="inlineStr">
         <x:is>
@@ -1557,10 +1557,10 @@
         </x:is>
       </x:c>
       <x:c r="E8" t="n">
-        <x:v>9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F8" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G8" t="inlineStr">
         <x:is>
@@ -1585,10 +1585,10 @@
         </x:is>
       </x:c>
       <x:c r="E9" t="n">
-        <x:v>29</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="F9" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G9" t="inlineStr">
         <x:is>
@@ -1613,10 +1613,10 @@
         </x:is>
       </x:c>
       <x:c r="E10" t="n">
-        <x:v>45</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="F10" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G10" t="inlineStr">
         <x:is>
@@ -1641,10 +1641,10 @@
         </x:is>
       </x:c>
       <x:c r="E11" t="n">
-        <x:v>19</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F11" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G11" t="inlineStr">
         <x:is>
@@ -1669,10 +1669,10 @@
         </x:is>
       </x:c>
       <x:c r="E12" t="n">
-        <x:v>17</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F12" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G12" t="inlineStr">
         <x:is>
@@ -1697,10 +1697,10 @@
         </x:is>
       </x:c>
       <x:c r="E13" t="n">
-        <x:v>41</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F13" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G13" t="inlineStr">
         <x:is>
@@ -1728,7 +1728,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F14" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G14" t="inlineStr">
         <x:is>
@@ -1753,7 +1753,7 @@
         </x:is>
       </x:c>
       <x:c r="E15" t="n">
-        <x:v>9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F15" t="n">
         <x:v>0</x:v>
@@ -1781,10 +1781,10 @@
         </x:is>
       </x:c>
       <x:c r="E16" t="n">
-        <x:v>35</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F16" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G16" t="inlineStr">
         <x:is>
@@ -1809,10 +1809,10 @@
         </x:is>
       </x:c>
       <x:c r="E17" t="n">
-        <x:v>35</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F17" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G17" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
fix: recalibrate placement grids for latest furniture sprites
</commit_message>
<xml_diff>
--- a/Excel/家具房间表.xlsx
+++ b/Excel/家具房间表.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="房间" sheetId="1" r:id="R189b7194a6704bed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网格" sheetId="2" r:id="R78b438265b7448e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="占用格" sheetId="3" r:id="R859aedb57e0d4072"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初始摆放" sheetId="4" r:id="R8884564ef8e2478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="房间" sheetId="1" r:id="R685e072adfb44ade"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网格" sheetId="2" r:id="R91604c8fc28d404b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="占用格" sheetId="3" r:id="Rbe582b84db2540e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初始摆放" sheetId="4" r:id="Rd82abcc1eda6441e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,6 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="0.###"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
+  </x:numFmts>
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
@@ -74,7 +78,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
@@ -84,6 +88,8 @@
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="常规" xfId="0"/>
@@ -952,307 +958,259 @@
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">living</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">壁挂</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" t="n">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="E3" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="F3" t="n">
+      <x:c r="A3" t="str">
+        <x:v>living</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>壁挂</x:v>
+      </x:c>
+      <x:c r="D3" s="5" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="E3" s="5" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F3" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G3" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H3" s="5" t="n">
+        <x:v>373</x:v>
+      </x:c>
+      <x:c r="I3" s="5" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="J3" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>living</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>地面</x:v>
+      </x:c>
+      <x:c r="D4" s="5" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="E4" s="5" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="G3" t="n">
+      <x:c r="F4" s="5" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="H3" t="n">
-        <x:v>316</x:v>
-      </x:c>
-      <x:c r="I3" t="n">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="J3" t="n">
+      <x:c r="G4" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H4" s="5" t="n">
+        <x:v>78.5</x:v>
+      </x:c>
+      <x:c r="I4" s="5" t="n">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="J4" s="5" t="n">
+        <x:v>0.603</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>bedroom</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>壁挂</x:v>
+      </x:c>
+      <x:c r="D5" s="5" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="E5" s="5" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F5" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G5" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H5" s="5" t="n">
+        <x:v>333.5</x:v>
+      </x:c>
+      <x:c r="I5" s="5" t="n">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="J5" s="5" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">living</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" t="n">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="E4" t="n">
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>bedroom</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>地面</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F6" s="5" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G6" s="5" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="F4" t="n">
+      <x:c r="H6" s="5" t="n">
+        <x:v>78.5</x:v>
+      </x:c>
+      <x:c r="I6" s="5" t="n">
+        <x:v>503</x:v>
+      </x:c>
+      <x:c r="J6" s="5" t="n">
+        <x:v>0.62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>kitchen</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>壁挂</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E7" s="5" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F7" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G7" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H7" s="5" t="n">
+        <x:v>645.5</x:v>
+      </x:c>
+      <x:c r="I7" s="5" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="J7" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>kitchen</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>地面</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="E8" s="5" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F8" s="5" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="G4" t="n">
-        <x:v>10.8</x:v>
-      </x:c>
-      <x:c r="H4" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="I4" t="n">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="J4" t="n">
-        <x:v>0.65</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bedroom</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">壁挂</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" t="n">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="E5" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F5" t="n">
+      <x:c r="G8" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H8" s="5" t="n">
+        <x:v>78.5</x:v>
+      </x:c>
+      <x:c r="I8" s="5" t="n">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="J8" s="5" t="n">
+        <x:v>0.56</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>study</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>壁挂</x:v>
+      </x:c>
+      <x:c r="D9" s="5" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E9" s="5" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="F9" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G9" s="5" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H9" s="5" t="n">
+        <x:v>310.5</x:v>
+      </x:c>
+      <x:c r="I9" s="5" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J9" s="5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>study</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>地面</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E10" s="5" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F10" s="5" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="G5" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H5" t="n">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="I5" t="n">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="J5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bedroom</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" t="n">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="E6" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F6" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G6" t="n">
-        <x:v>10.5</x:v>
-      </x:c>
-      <x:c r="H6" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="I6" t="n">
-        <x:v>530</x:v>
-      </x:c>
-      <x:c r="J6" t="n">
-        <x:v>0.74</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kitchen</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">壁挂</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="E7" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="F7" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G7" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H7" t="n">
-        <x:v>562</x:v>
-      </x:c>
-      <x:c r="I7" t="n">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="J7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kitchen</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" t="n">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="E8" t="n">
+      <x:c r="G10" s="5" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="F8" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G8" t="n">
-        <x:v>10.4</x:v>
-      </x:c>
-      <x:c r="H8" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="I8" t="n">
-        <x:v>502</x:v>
-      </x:c>
-      <x:c r="J8" t="n">
-        <x:v>0.65</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">study</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">壁挂</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" t="n">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="E9" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="F9" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G9" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H9" t="n">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="I9" t="n">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="J9" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">study</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">地面</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" t="n">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="E10" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="F10" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="G10" t="n">
-        <x:v>10.05</x:v>
-      </x:c>
-      <x:c r="H10" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="I10" t="n">
-        <x:v>502</x:v>
-      </x:c>
-      <x:c r="J10" t="n">
-        <x:v>0.88</x:v>
+      <x:c r="H10" s="5" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="I10" s="5" t="n">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="J10" s="5" t="n">
+        <x:v>0.69</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1401,424 +1359,346 @@
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">living</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">landscape_poster_02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="F3" t="n">
+      <x:c r="A3" t="str">
+        <x:v>living</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>landscape_poster_02</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="D3"/>
+      <x:c r="E3" s="6" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
+      <x:c r="G3" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">living</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">hanging_plant_01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="F4" t="n">
+      <x:c r="A4" t="str">
+        <x:v>living</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>hanging_plant_01</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="D4"/>
+      <x:c r="E4" s="6" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
+      <x:c r="G4" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">living</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">armchair_01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" t="n">
+      <x:c r="A5" t="str">
+        <x:v>living</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>armchair_01</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D5"/>
+      <x:c r="E5" s="6" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="F5" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
+      <x:c r="F5" s="6" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">living</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">round_table_01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="F6" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
+      <x:c r="A6" t="str">
+        <x:v>living</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>round_table_01</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D6"/>
+      <x:c r="E6" s="6" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bedroom</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">landscape_poster_03</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F7" t="n">
+      <x:c r="A7" t="str">
+        <x:v>bedroom</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>landscape_poster_03</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="D7"/>
+      <x:c r="E7" s="6" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>bedroom</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>single_sofa_02</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D8"/>
+      <x:c r="E8" s="6" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>bedroom</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>cat_sofa_01</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D9"/>
+      <x:c r="E9" s="6" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>bedroom</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>monstera_01</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D10"/>
+      <x:c r="E10" s="6" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>kitchen</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>vintage_square_clock_02</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="D11"/>
+      <x:c r="E11" s="6" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>kitchen</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>round_table_02</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D12"/>
+      <x:c r="E12" s="6" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>kitchen</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>potted_plant_01</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D13"/>
+      <x:c r="E13" s="6" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bedroom</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">single_sofa_02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E8" t="n">
+      <x:c r="G13" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>study</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>round_table_03</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D14"/>
+      <x:c r="E14" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>study</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>potted_plant_02</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D15"/>
+      <x:c r="E15" s="6" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="F8" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bedroom</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cat_sofa_01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" t="n">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="F9" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bedroom</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">monstera_01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" t="n">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="F10" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kitchen</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">vintage_square_clock_02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E11" t="n">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="F11" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="G11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kitchen</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">round_table_02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" t="n">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="F12" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kitchen</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">potted_plant_01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E13" t="n">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="F13" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">study</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">round_table_03</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E14" t="n">
+      <x:c r="F15" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F14" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">study</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">potted_plant_02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E15" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="F15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
+      <x:c r="G15" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">study</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">vintage_square_clock_03</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">wall</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E16" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="F16" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="G16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
+      <x:c r="A16" t="str">
+        <x:v>study</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>vintage_square_clock_03</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>wall</x:v>
+      </x:c>
+      <x:c r="D16"/>
+      <x:c r="E16" s="6" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">study</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">single_sofa_04</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">floor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E17" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="F17" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">否</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A17" t="str">
+        <x:v>study</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>single_sofa_04</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>floor</x:v>
+      </x:c>
+      <x:c r="D17"/>
+      <x:c r="E17" s="6" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>否</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18" s="6"/>
+      <x:c r="F18" s="6"/>
+      <x:c r="G18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19" s="6"/>
+      <x:c r="F19" s="6"/>
+      <x:c r="G19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20" s="6"/>
+      <x:c r="F20" s="6"/>
+      <x:c r="G20"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: align night room art with placement geometry
</commit_message>
<xml_diff>
--- a/Excel/家具房间表.xlsx
+++ b/Excel/家具房间表.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="房间" sheetId="1" r:id="R685e072adfb44ade"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网格" sheetId="2" r:id="R91604c8fc28d404b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="占用格" sheetId="3" r:id="Rbe582b84db2540e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初始摆放" sheetId="4" r:id="Rd82abcc1eda6441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="房间" sheetId="1" r:id="R41d1feeeb45a4a70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网格" sheetId="2" r:id="R42ea7346d5c541ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="占用格" sheetId="3" r:id="R7f472517549f4be2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初始摆放" sheetId="4" r:id="R9ac6f38ed209449f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -644,13 +644,13 @@
         <x:v>0.7943</x:v>
       </x:c>
       <x:c r="R3" t="n">
-        <x:v>0.8015</x:v>
+        <x:v>0.7943</x:v>
       </x:c>
       <x:c r="S3" t="n">
-        <x:v>0.99</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T3" t="n">
-        <x:v>13.2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -706,13 +706,13 @@
         <x:v>0.832</x:v>
       </x:c>
       <x:c r="R4" t="n">
-        <x:v>0.8931</x:v>
+        <x:v>0.832</x:v>
       </x:c>
       <x:c r="S4" t="n">
-        <x:v>1.062</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T4" t="n">
-        <x:v>47.9</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -768,13 +768,13 @@
         <x:v>0.7853</x:v>
       </x:c>
       <x:c r="R5" t="n">
-        <x:v>0.7825</x:v>
+        <x:v>0.7853</x:v>
       </x:c>
       <x:c r="S5" t="n">
-        <x:v>1.066</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="T5" t="n">
-        <x:v>171.1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -830,7 +830,7 @@
         <x:v>0.8</x:v>
       </x:c>
       <x:c r="R6" t="n">
-        <x:v>0.8753</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="S6" t="n">
         <x:v>1</x:v>

</xml_diff>